<commit_message>
updating the excel files
</commit_message>
<xml_diff>
--- a/BOND_EQT/reg_HS Tech.xlsx
+++ b/BOND_EQT/reg_HS Tech.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c060ac0a7f9c7ae2/main/CRAMC_Desktop/EU/BOND_EQT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{2773DC52-B2E1-442E-8E9F-479DDE4DEB2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8BCB6FC-3F1A-4A83-B7BE-55B77E4F66C0}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{2773DC52-B2E1-442E-8E9F-479DDE4DEB2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCCE39A4-F6E1-4578-B0D1-DC69D144E713}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="480" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="480" windowWidth="16440" windowHeight="28440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -130,21 +130,21 @@
       <tp t="e">
         <v>#N/A</v>
         <stp/>
-        <stp>BDH|14049501234159561198</stp>
+        <stp>BDH|12960302437871177505</stp>
         <tr r="C1" s="2"/>
+      </tp>
+    </main>
+    <main first="bofaddin.rtdserver">
+      <tp t="e">
+        <v>#N/A</v>
+        <stp/>
+        <stp>BDH|3251234060618079766</stp>
+        <tr r="D1" s="2"/>
       </tp>
       <tp t="e">
         <v>#N/A</v>
         <stp/>
-        <stp>BDH|12379947721503079785</stp>
-        <tr r="D1" s="2"/>
-      </tp>
-    </main>
-    <main first="bofaddin.rtdserver">
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|5880802984461791641</stp>
+        <stp>BDH|279743278180750885</stp>
         <tr r="A1" s="2"/>
       </tp>
     </main>
@@ -419,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1872"/>
+  <dimension ref="A1:C1900"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -20666,7 +20666,7 @@
       </c>
     </row>
     <row r="1841" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1841">
+      <c r="A1841" s="1">
         <v>45878</v>
       </c>
       <c r="B1841">
@@ -20677,7 +20677,7 @@
       </c>
     </row>
     <row r="1842" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1842">
+      <c r="A1842" s="1">
         <v>45879</v>
       </c>
       <c r="B1842">
@@ -20688,7 +20688,7 @@
       </c>
     </row>
     <row r="1843" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1843">
+      <c r="A1843" s="1">
         <v>45880</v>
       </c>
       <c r="B1843">
@@ -20699,7 +20699,7 @@
       </c>
     </row>
     <row r="1844" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1844">
+      <c r="A1844" s="1">
         <v>45881</v>
       </c>
       <c r="B1844">
@@ -20710,7 +20710,7 @@
       </c>
     </row>
     <row r="1845" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1845">
+      <c r="A1845" s="1">
         <v>45882</v>
       </c>
       <c r="B1845">
@@ -20721,7 +20721,7 @@
       </c>
     </row>
     <row r="1846" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1846">
+      <c r="A1846" s="1">
         <v>45883</v>
       </c>
       <c r="B1846">
@@ -20732,7 +20732,7 @@
       </c>
     </row>
     <row r="1847" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1847">
+      <c r="A1847" s="1">
         <v>45884</v>
       </c>
       <c r="B1847">
@@ -20743,7 +20743,7 @@
       </c>
     </row>
     <row r="1848" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1848">
+      <c r="A1848" s="1">
         <v>45885</v>
       </c>
       <c r="B1848">
@@ -20754,7 +20754,7 @@
       </c>
     </row>
     <row r="1849" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1849">
+      <c r="A1849" s="1">
         <v>45886</v>
       </c>
       <c r="B1849">
@@ -20765,7 +20765,7 @@
       </c>
     </row>
     <row r="1850" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1850">
+      <c r="A1850" s="1">
         <v>45887</v>
       </c>
       <c r="B1850">
@@ -20776,7 +20776,7 @@
       </c>
     </row>
     <row r="1851" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1851">
+      <c r="A1851" s="1">
         <v>45888</v>
       </c>
       <c r="B1851">
@@ -20787,7 +20787,7 @@
       </c>
     </row>
     <row r="1852" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1852">
+      <c r="A1852" s="1">
         <v>45889</v>
       </c>
       <c r="B1852">
@@ -20798,7 +20798,7 @@
       </c>
     </row>
     <row r="1853" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1853">
+      <c r="A1853" s="1">
         <v>45890</v>
       </c>
       <c r="B1853">
@@ -20809,7 +20809,7 @@
       </c>
     </row>
     <row r="1854" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1854">
+      <c r="A1854" s="1">
         <v>45891</v>
       </c>
       <c r="B1854">
@@ -20820,7 +20820,7 @@
       </c>
     </row>
     <row r="1855" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1855">
+      <c r="A1855" s="1">
         <v>45892</v>
       </c>
       <c r="B1855">
@@ -20831,7 +20831,7 @@
       </c>
     </row>
     <row r="1856" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1856">
+      <c r="A1856" s="1">
         <v>45893</v>
       </c>
       <c r="B1856">
@@ -20842,7 +20842,7 @@
       </c>
     </row>
     <row r="1857" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1857">
+      <c r="A1857" s="1">
         <v>45894</v>
       </c>
       <c r="B1857">
@@ -20853,7 +20853,7 @@
       </c>
     </row>
     <row r="1858" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1858">
+      <c r="A1858" s="1">
         <v>45895</v>
       </c>
       <c r="B1858">
@@ -20864,7 +20864,7 @@
       </c>
     </row>
     <row r="1859" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1859">
+      <c r="A1859" s="1">
         <v>45896</v>
       </c>
       <c r="B1859">
@@ -20875,7 +20875,7 @@
       </c>
     </row>
     <row r="1860" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1860">
+      <c r="A1860" s="1">
         <v>45897</v>
       </c>
       <c r="B1860">
@@ -20886,7 +20886,7 @@
       </c>
     </row>
     <row r="1861" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1861">
+      <c r="A1861" s="1">
         <v>45898</v>
       </c>
       <c r="B1861">
@@ -20897,7 +20897,7 @@
       </c>
     </row>
     <row r="1862" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1862">
+      <c r="A1862" s="1">
         <v>45899</v>
       </c>
       <c r="B1862">
@@ -20908,7 +20908,7 @@
       </c>
     </row>
     <row r="1863" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1863">
+      <c r="A1863" s="1">
         <v>45900</v>
       </c>
       <c r="B1863">
@@ -20919,7 +20919,7 @@
       </c>
     </row>
     <row r="1864" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1864">
+      <c r="A1864" s="1">
         <v>45901</v>
       </c>
       <c r="B1864">
@@ -20930,7 +20930,7 @@
       </c>
     </row>
     <row r="1865" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1865">
+      <c r="A1865" s="1">
         <v>45902</v>
       </c>
       <c r="B1865">
@@ -20941,7 +20941,7 @@
       </c>
     </row>
     <row r="1866" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1866">
+      <c r="A1866" s="1">
         <v>45903</v>
       </c>
       <c r="B1866">
@@ -20952,7 +20952,7 @@
       </c>
     </row>
     <row r="1867" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1867">
+      <c r="A1867" s="1">
         <v>45904</v>
       </c>
       <c r="B1867">
@@ -20963,7 +20963,7 @@
       </c>
     </row>
     <row r="1868" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1868">
+      <c r="A1868" s="1">
         <v>45905</v>
       </c>
       <c r="B1868">
@@ -20974,7 +20974,7 @@
       </c>
     </row>
     <row r="1869" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1869">
+      <c r="A1869" s="1">
         <v>45906</v>
       </c>
       <c r="B1869">
@@ -20985,7 +20985,7 @@
       </c>
     </row>
     <row r="1870" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1870">
+      <c r="A1870" s="1">
         <v>45907</v>
       </c>
       <c r="B1870">
@@ -20996,7 +20996,7 @@
       </c>
     </row>
     <row r="1871" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1871">
+      <c r="A1871" s="1">
         <v>45908</v>
       </c>
       <c r="B1871">
@@ -21007,7 +21007,7 @@
       </c>
     </row>
     <row r="1872" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1872">
+      <c r="A1872" s="1">
         <v>45909</v>
       </c>
       <c r="B1872">
@@ -21015,6 +21015,314 @@
       </c>
       <c r="C1872">
         <v>-2.2865000000000002</v>
+      </c>
+    </row>
+    <row r="1873" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1873" s="1">
+        <v>45910</v>
+      </c>
+      <c r="B1873">
+        <v>5902.69</v>
+      </c>
+      <c r="C1873">
+        <v>-2.2214</v>
+      </c>
+    </row>
+    <row r="1874" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1874" s="1">
+        <v>45911</v>
+      </c>
+      <c r="B1874">
+        <v>5888.77</v>
+      </c>
+      <c r="C1874">
+        <v>-2.2136</v>
+      </c>
+    </row>
+    <row r="1875" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1875" s="1">
+        <v>45912</v>
+      </c>
+      <c r="B1875">
+        <v>5989.27</v>
+      </c>
+      <c r="C1875">
+        <v>-2.2623000000000002</v>
+      </c>
+    </row>
+    <row r="1876" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1876" s="1">
+        <v>45913</v>
+      </c>
+      <c r="B1876">
+        <v>5989.27</v>
+      </c>
+      <c r="C1876">
+        <v>-2.2623000000000002</v>
+      </c>
+    </row>
+    <row r="1877" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1877" s="1">
+        <v>45914</v>
+      </c>
+      <c r="B1877">
+        <v>5989.27</v>
+      </c>
+      <c r="C1877">
+        <v>-2.2623000000000002</v>
+      </c>
+    </row>
+    <row r="1878" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1878" s="1">
+        <v>45915</v>
+      </c>
+      <c r="B1878">
+        <v>6043.61</v>
+      </c>
+      <c r="C1878">
+        <v>-2.2364999999999995</v>
+      </c>
+    </row>
+    <row r="1879" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1879" s="1">
+        <v>45916</v>
+      </c>
+      <c r="B1879">
+        <v>6077.66</v>
+      </c>
+      <c r="C1879">
+        <v>-2.2408999999999999</v>
+      </c>
+    </row>
+    <row r="1880" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1880" s="1">
+        <v>45917</v>
+      </c>
+      <c r="B1880">
+        <v>6334.24</v>
+      </c>
+      <c r="C1880">
+        <v>-2.3162000000000003</v>
+      </c>
+    </row>
+    <row r="1881" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1881" s="1">
+        <v>45918</v>
+      </c>
+      <c r="B1881">
+        <v>6271.22</v>
+      </c>
+      <c r="C1881">
+        <v>-2.3224</v>
+      </c>
+    </row>
+    <row r="1882" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1882" s="1">
+        <v>45919</v>
+      </c>
+      <c r="B1882">
+        <v>6294.42</v>
+      </c>
+      <c r="C1882">
+        <v>-2.3293999999999997</v>
+      </c>
+    </row>
+    <row r="1883" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1883" s="1">
+        <v>45920</v>
+      </c>
+      <c r="B1883">
+        <v>6294.42</v>
+      </c>
+      <c r="C1883">
+        <v>-2.3293999999999997</v>
+      </c>
+    </row>
+    <row r="1884" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1884" s="1">
+        <v>45921</v>
+      </c>
+      <c r="B1884">
+        <v>6294.42</v>
+      </c>
+      <c r="C1884">
+        <v>-2.3293999999999997</v>
+      </c>
+    </row>
+    <row r="1885" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1885" s="1">
+        <v>45922</v>
+      </c>
+      <c r="B1885">
+        <v>6257.91</v>
+      </c>
+      <c r="C1885">
+        <v>-2.3547000000000002</v>
+      </c>
+    </row>
+    <row r="1886" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1886" s="1">
+        <v>45923</v>
+      </c>
+      <c r="B1886">
+        <v>6167.06</v>
+      </c>
+      <c r="C1886">
+        <v>-2.3040999999999996</v>
+      </c>
+    </row>
+    <row r="1887" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1887" s="1">
+        <v>45924</v>
+      </c>
+      <c r="B1887">
+        <v>6323.15</v>
+      </c>
+      <c r="C1887">
+        <v>-2.2416</v>
+      </c>
+    </row>
+    <row r="1888" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1888" s="1">
+        <v>45925</v>
+      </c>
+      <c r="B1888">
+        <v>6379.19</v>
+      </c>
+      <c r="C1888">
+        <v>-2.2768000000000006</v>
+      </c>
+    </row>
+    <row r="1889" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1889" s="1">
+        <v>45926</v>
+      </c>
+      <c r="B1889">
+        <v>6195.11</v>
+      </c>
+      <c r="C1889">
+        <v>-2.2875000000000005</v>
+      </c>
+    </row>
+    <row r="1890" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1890" s="1">
+        <v>45927</v>
+      </c>
+      <c r="B1890">
+        <v>6195.11</v>
+      </c>
+      <c r="C1890">
+        <v>-2.2875000000000005</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1891" s="1">
+        <v>45928</v>
+      </c>
+      <c r="B1891">
+        <v>6195.11</v>
+      </c>
+      <c r="C1891">
+        <v>-2.2875000000000005</v>
+      </c>
+    </row>
+    <row r="1892" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1892" s="1">
+        <v>45929</v>
+      </c>
+      <c r="B1892">
+        <v>6324.25</v>
+      </c>
+      <c r="C1892">
+        <v>-2.2416999999999998</v>
+      </c>
+    </row>
+    <row r="1893" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1893" s="1">
+        <v>45930</v>
+      </c>
+      <c r="B1893">
+        <v>6465.66</v>
+      </c>
+      <c r="C1893">
+        <v>-2.2792999999999997</v>
+      </c>
+    </row>
+    <row r="1894" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1894" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B1894">
+        <v>6465.66</v>
+      </c>
+      <c r="C1894">
+        <v>-2.2270999999999996</v>
+      </c>
+    </row>
+    <row r="1895" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1895" s="1">
+        <v>45932</v>
+      </c>
+      <c r="B1895">
+        <v>6682.86</v>
+      </c>
+      <c r="C1895">
+        <v>-2.2117</v>
+      </c>
+    </row>
+    <row r="1896" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1896" s="1">
+        <v>45933</v>
+      </c>
+      <c r="B1896">
+        <v>6622.85</v>
+      </c>
+      <c r="C1896">
+        <v>-2.2482000000000002</v>
+      </c>
+    </row>
+    <row r="1897" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1897" s="1">
+        <v>45934</v>
+      </c>
+      <c r="B1897">
+        <v>6622.85</v>
+      </c>
+      <c r="C1897">
+        <v>-2.2482000000000002</v>
+      </c>
+    </row>
+    <row r="1898" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1898" s="1">
+        <v>45935</v>
+      </c>
+      <c r="B1898">
+        <v>6622.85</v>
+      </c>
+      <c r="C1898">
+        <v>-2.2482000000000002</v>
+      </c>
+    </row>
+    <row r="1899" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1899" s="1">
+        <v>45936</v>
+      </c>
+      <c r="B1899">
+        <v>6550.3</v>
+      </c>
+      <c r="C1899">
+        <v>-2.2810000000000001</v>
+      </c>
+    </row>
+    <row r="1900" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1900" s="1">
+        <v>45937</v>
+      </c>
+      <c r="B1900">
+        <v>6550.3</v>
+      </c>
+      <c r="C1900">
+        <v>-2.2520000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -21024,26 +21332,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C44AB31A-70CE-4A6E-A84E-7592026AAEFA}">
-  <dimension ref="A1:E1873"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E1899"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="0" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="9.140625" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" cm="1">
-        <f t="array" ref="A1:B1871">_xll.BDH("HSTECH Index", "PX_LAST", "7/27/2020", "9/9/2025", "Days", "C", "BEST_FPERIOD_OVERRIDE", "1BF")</f>
+        <f t="array" ref="A1:B1899">_xll.BDH("HSTECH Index", "PX_LAST", "7/27/2020", "10/7/2025", "Days", "C", "BEST_FPERIOD_OVERRIDE", "1BF")</f>
         <v>44039</v>
       </c>
       <c r="B1">
         <v>6774.78</v>
       </c>
       <c r="C1" cm="1">
-        <f t="array" ref="C1:C1871">_xll.BDH("GCNY10YR Index", "PX_LAST", "7/27/2020", "9/9/2025", "Days", "C", "Dates", "Hide")</f>
+        <f t="array" ref="C1:C1899">_xll.BDH("GCNY10YR Index", "PX_LAST", "7/27/2020", "10/7/2025", "Days", "C", "Dates", "Hide")</f>
         <v>2.8959999999999999</v>
       </c>
       <c r="D1" cm="1">
-        <f t="array" ref="D1:D1871">_xll.BDH("USGG10YR Index", "PX_LAST", "7/27/2020", "9/9/2025", "Days", "C", "Dates", "Hide")</f>
+        <f t="array" ref="D1:D1899">_xll.BDH("USGG10YR Index", "PX_LAST", "7/27/2020", "10/7/2025", "Days", "C", "Dates", "Hide")</f>
         <v>0.61509999999999998</v>
       </c>
       <c r="E1">
@@ -54473,7 +54783,7 @@
         <v>4.2343000000000002</v>
       </c>
       <c r="E1858">
-        <f t="shared" ref="E1858:E1871" si="29">C1858-D1858</f>
+        <f t="shared" ref="E1858:E1899" si="29">C1858-D1858</f>
         <v>-2.4643000000000002</v>
       </c>
     </row>
@@ -54712,10 +55022,508 @@
       </c>
     </row>
     <row r="1872" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1872" s="1"/>
-    </row>
-    <row r="1873" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1873" s="1"/>
+      <c r="A1872" s="1">
+        <v>45910</v>
+      </c>
+      <c r="B1872">
+        <v>5902.69</v>
+      </c>
+      <c r="C1872">
+        <v>1.8240000000000001</v>
+      </c>
+      <c r="D1872">
+        <v>4.0453999999999999</v>
+      </c>
+      <c r="E1872">
+        <f t="shared" si="29"/>
+        <v>-2.2214</v>
+      </c>
+    </row>
+    <row r="1873" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1873" s="1">
+        <v>45911</v>
+      </c>
+      <c r="B1873">
+        <v>5888.77</v>
+      </c>
+      <c r="C1873">
+        <v>1.8069999999999999</v>
+      </c>
+      <c r="D1873">
+        <v>4.0206</v>
+      </c>
+      <c r="E1873">
+        <f t="shared" si="29"/>
+        <v>-2.2136</v>
+      </c>
+    </row>
+    <row r="1874" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1874" s="1">
+        <v>45912</v>
+      </c>
+      <c r="B1874">
+        <v>5989.27</v>
+      </c>
+      <c r="C1874">
+        <v>1.802</v>
+      </c>
+      <c r="D1874">
+        <v>4.0643000000000002</v>
+      </c>
+      <c r="E1874">
+        <f t="shared" si="29"/>
+        <v>-2.2623000000000002</v>
+      </c>
+    </row>
+    <row r="1875" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1875" s="1">
+        <v>45913</v>
+      </c>
+      <c r="B1875">
+        <v>5989.27</v>
+      </c>
+      <c r="C1875">
+        <v>1.802</v>
+      </c>
+      <c r="D1875">
+        <v>4.0643000000000002</v>
+      </c>
+      <c r="E1875">
+        <f t="shared" si="29"/>
+        <v>-2.2623000000000002</v>
+      </c>
+    </row>
+    <row r="1876" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1876" s="1">
+        <v>45914</v>
+      </c>
+      <c r="B1876">
+        <v>5989.27</v>
+      </c>
+      <c r="C1876">
+        <v>1.802</v>
+      </c>
+      <c r="D1876">
+        <v>4.0643000000000002</v>
+      </c>
+      <c r="E1876">
+        <f t="shared" si="29"/>
+        <v>-2.2623000000000002</v>
+      </c>
+    </row>
+    <row r="1877" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1877" s="1">
+        <v>45915</v>
+      </c>
+      <c r="B1877">
+        <v>6043.61</v>
+      </c>
+      <c r="C1877">
+        <v>1.8009999999999999</v>
+      </c>
+      <c r="D1877">
+        <v>4.0374999999999996</v>
+      </c>
+      <c r="E1877">
+        <f t="shared" si="29"/>
+        <v>-2.2364999999999995</v>
+      </c>
+    </row>
+    <row r="1878" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1878" s="1">
+        <v>45916</v>
+      </c>
+      <c r="B1878">
+        <v>6077.66</v>
+      </c>
+      <c r="C1878">
+        <v>1.7869999999999999</v>
+      </c>
+      <c r="D1878">
+        <v>4.0278999999999998</v>
+      </c>
+      <c r="E1878">
+        <f t="shared" si="29"/>
+        <v>-2.2408999999999999</v>
+      </c>
+    </row>
+    <row r="1879" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1879" s="1">
+        <v>45917</v>
+      </c>
+      <c r="B1879">
+        <v>6334.24</v>
+      </c>
+      <c r="C1879">
+        <v>1.7709999999999999</v>
+      </c>
+      <c r="D1879">
+        <v>4.0872000000000002</v>
+      </c>
+      <c r="E1879">
+        <f t="shared" si="29"/>
+        <v>-2.3162000000000003</v>
+      </c>
+    </row>
+    <row r="1880" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1880" s="1">
+        <v>45918</v>
+      </c>
+      <c r="B1880">
+        <v>6271.22</v>
+      </c>
+      <c r="C1880">
+        <v>1.782</v>
+      </c>
+      <c r="D1880">
+        <v>4.1044</v>
+      </c>
+      <c r="E1880">
+        <f t="shared" si="29"/>
+        <v>-2.3224</v>
+      </c>
+    </row>
+    <row r="1881" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1881" s="1">
+        <v>45919</v>
+      </c>
+      <c r="B1881">
+        <v>6294.42</v>
+      </c>
+      <c r="C1881">
+        <v>1.798</v>
+      </c>
+      <c r="D1881">
+        <v>4.1273999999999997</v>
+      </c>
+      <c r="E1881">
+        <f t="shared" si="29"/>
+        <v>-2.3293999999999997</v>
+      </c>
+    </row>
+    <row r="1882" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1882" s="1">
+        <v>45920</v>
+      </c>
+      <c r="B1882">
+        <v>6294.42</v>
+      </c>
+      <c r="C1882">
+        <v>1.798</v>
+      </c>
+      <c r="D1882">
+        <v>4.1273999999999997</v>
+      </c>
+      <c r="E1882">
+        <f t="shared" si="29"/>
+        <v>-2.3293999999999997</v>
+      </c>
+    </row>
+    <row r="1883" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1883" s="1">
+        <v>45921</v>
+      </c>
+      <c r="B1883">
+        <v>6294.42</v>
+      </c>
+      <c r="C1883">
+        <v>1.798</v>
+      </c>
+      <c r="D1883">
+        <v>4.1273999999999997</v>
+      </c>
+      <c r="E1883">
+        <f t="shared" si="29"/>
+        <v>-2.3293999999999997</v>
+      </c>
+    </row>
+    <row r="1884" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1884" s="1">
+        <v>45922</v>
+      </c>
+      <c r="B1884">
+        <v>6257.91</v>
+      </c>
+      <c r="C1884">
+        <v>1.792</v>
+      </c>
+      <c r="D1884">
+        <v>4.1467000000000001</v>
+      </c>
+      <c r="E1884">
+        <f t="shared" si="29"/>
+        <v>-2.3547000000000002</v>
+      </c>
+    </row>
+    <row r="1885" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1885" s="1">
+        <v>45923</v>
+      </c>
+      <c r="B1885">
+        <v>6167.06</v>
+      </c>
+      <c r="C1885">
+        <v>1.802</v>
+      </c>
+      <c r="D1885">
+        <v>4.1060999999999996</v>
+      </c>
+      <c r="E1885">
+        <f t="shared" si="29"/>
+        <v>-2.3040999999999996</v>
+      </c>
+    </row>
+    <row r="1886" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1886" s="1">
+        <v>45924</v>
+      </c>
+      <c r="B1886">
+        <v>6323.15</v>
+      </c>
+      <c r="C1886">
+        <v>1.905</v>
+      </c>
+      <c r="D1886">
+        <v>4.1466000000000003</v>
+      </c>
+      <c r="E1886">
+        <f t="shared" si="29"/>
+        <v>-2.2416</v>
+      </c>
+    </row>
+    <row r="1887" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1887" s="1">
+        <v>45925</v>
+      </c>
+      <c r="B1887">
+        <v>6379.19</v>
+      </c>
+      <c r="C1887">
+        <v>1.893</v>
+      </c>
+      <c r="D1887">
+        <v>4.1698000000000004</v>
+      </c>
+      <c r="E1887">
+        <f t="shared" si="29"/>
+        <v>-2.2768000000000006</v>
+      </c>
+    </row>
+    <row r="1888" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1888" s="1">
+        <v>45926</v>
+      </c>
+      <c r="B1888">
+        <v>6195.11</v>
+      </c>
+      <c r="C1888">
+        <v>1.8879999999999999</v>
+      </c>
+      <c r="D1888">
+        <v>4.1755000000000004</v>
+      </c>
+      <c r="E1888">
+        <f t="shared" si="29"/>
+        <v>-2.2875000000000005</v>
+      </c>
+    </row>
+    <row r="1889" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1889" s="1">
+        <v>45927</v>
+      </c>
+      <c r="B1889">
+        <v>6195.11</v>
+      </c>
+      <c r="C1889">
+        <v>1.8879999999999999</v>
+      </c>
+      <c r="D1889">
+        <v>4.1755000000000004</v>
+      </c>
+      <c r="E1889">
+        <f t="shared" si="29"/>
+        <v>-2.2875000000000005</v>
+      </c>
+    </row>
+    <row r="1890" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1890" s="1">
+        <v>45928</v>
+      </c>
+      <c r="B1890">
+        <v>6195.11</v>
+      </c>
+      <c r="C1890">
+        <v>1.8879999999999999</v>
+      </c>
+      <c r="D1890">
+        <v>4.1755000000000004</v>
+      </c>
+      <c r="E1890">
+        <f t="shared" si="29"/>
+        <v>-2.2875000000000005</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1891" s="1">
+        <v>45929</v>
+      </c>
+      <c r="B1891">
+        <v>6324.25</v>
+      </c>
+      <c r="C1891">
+        <v>1.897</v>
+      </c>
+      <c r="D1891">
+        <v>4.1387</v>
+      </c>
+      <c r="E1891">
+        <f t="shared" si="29"/>
+        <v>-2.2416999999999998</v>
+      </c>
+    </row>
+    <row r="1892" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1892" s="1">
+        <v>45930</v>
+      </c>
+      <c r="B1892">
+        <v>6465.66</v>
+      </c>
+      <c r="C1892">
+        <v>1.871</v>
+      </c>
+      <c r="D1892">
+        <v>4.1502999999999997</v>
+      </c>
+      <c r="E1892">
+        <f t="shared" si="29"/>
+        <v>-2.2792999999999997</v>
+      </c>
+    </row>
+    <row r="1893" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1893" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B1893">
+        <v>6465.66</v>
+      </c>
+      <c r="C1893">
+        <v>1.871</v>
+      </c>
+      <c r="D1893">
+        <v>4.0980999999999996</v>
+      </c>
+      <c r="E1893">
+        <f t="shared" si="29"/>
+        <v>-2.2270999999999996</v>
+      </c>
+    </row>
+    <row r="1894" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1894" s="1">
+        <v>45932</v>
+      </c>
+      <c r="B1894">
+        <v>6682.86</v>
+      </c>
+      <c r="C1894">
+        <v>1.871</v>
+      </c>
+      <c r="D1894">
+        <v>4.0827</v>
+      </c>
+      <c r="E1894">
+        <f t="shared" si="29"/>
+        <v>-2.2117</v>
+      </c>
+    </row>
+    <row r="1895" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1895" s="1">
+        <v>45933</v>
+      </c>
+      <c r="B1895">
+        <v>6622.85</v>
+      </c>
+      <c r="C1895">
+        <v>1.871</v>
+      </c>
+      <c r="D1895">
+        <v>4.1192000000000002</v>
+      </c>
+      <c r="E1895">
+        <f t="shared" si="29"/>
+        <v>-2.2482000000000002</v>
+      </c>
+    </row>
+    <row r="1896" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1896" s="1">
+        <v>45934</v>
+      </c>
+      <c r="B1896">
+        <v>6622.85</v>
+      </c>
+      <c r="C1896">
+        <v>1.871</v>
+      </c>
+      <c r="D1896">
+        <v>4.1192000000000002</v>
+      </c>
+      <c r="E1896">
+        <f t="shared" si="29"/>
+        <v>-2.2482000000000002</v>
+      </c>
+    </row>
+    <row r="1897" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1897" s="1">
+        <v>45935</v>
+      </c>
+      <c r="B1897">
+        <v>6622.85</v>
+      </c>
+      <c r="C1897">
+        <v>1.871</v>
+      </c>
+      <c r="D1897">
+        <v>4.1192000000000002</v>
+      </c>
+      <c r="E1897">
+        <f t="shared" si="29"/>
+        <v>-2.2482000000000002</v>
+      </c>
+    </row>
+    <row r="1898" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1898" s="1">
+        <v>45936</v>
+      </c>
+      <c r="B1898">
+        <v>6550.3</v>
+      </c>
+      <c r="C1898">
+        <v>1.871</v>
+      </c>
+      <c r="D1898">
+        <v>4.1520000000000001</v>
+      </c>
+      <c r="E1898">
+        <f t="shared" si="29"/>
+        <v>-2.2810000000000001</v>
+      </c>
+    </row>
+    <row r="1899" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1899" s="1">
+        <v>45937</v>
+      </c>
+      <c r="B1899">
+        <v>6550.3</v>
+      </c>
+      <c r="C1899">
+        <v>1.871</v>
+      </c>
+      <c r="D1899">
+        <v>4.1230000000000002</v>
+      </c>
+      <c r="E1899">
+        <f t="shared" si="29"/>
+        <v>-2.2520000000000002</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C275">

</xml_diff>